<commit_message>
added the path location in cleaned data.csv and in report generating folder analysis report file and topproducts salespersons files
</commit_message>
<xml_diff>
--- a/Sales_Analysis_Report.xlsx
+++ b/Sales_Analysis_Report.xlsx
@@ -1,144 +1,42 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29127"/>
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Admin\Desktop\Final Project\"/>
-    </mc:Choice>
-  </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BCF270FD-716C-4396-94CE-9BAF8633379F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <workbookProtection/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="26160" windowHeight="13170" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Overall Summary" sheetId="1" r:id="rId1"/>
-    <sheet name="Region Summary" sheetId="2" r:id="rId2"/>
-    <sheet name="Top Products" sheetId="3" r:id="rId3"/>
-    <sheet name="Top Salespersons" sheetId="4" r:id="rId4"/>
-    <sheet name="Daily Totals" sheetId="5" r:id="rId5"/>
-    <sheet name="Monthly Totals" sheetId="6" r:id="rId6"/>
+    <sheet name="Overall Summary" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Region Summary" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Top Products" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Top Salespersons" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Daily Totals" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="Monthly Totals" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
-  <calcPr calcId="0"/>
+  <definedNames/>
+  <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
-<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="41" uniqueCount="31">
-  <si>
-    <t>Metric</t>
-  </si>
-  <si>
-    <t>Value</t>
-  </si>
-  <si>
-    <t>Total Revenue</t>
-  </si>
-  <si>
-    <t>Total Quantity Sold</t>
-  </si>
-  <si>
-    <t>Unique Orders</t>
-  </si>
-  <si>
-    <t>Region</t>
-  </si>
-  <si>
-    <t>Total_Revenue</t>
-  </si>
-  <si>
-    <t>Total_Quantity</t>
-  </si>
-  <si>
-    <t>Total_Orders</t>
-  </si>
-  <si>
-    <t>West</t>
-  </si>
-  <si>
-    <t>East</t>
-  </si>
-  <si>
-    <t>North</t>
-  </si>
-  <si>
-    <t>South</t>
-  </si>
-  <si>
-    <t xml:space="preserve"> south </t>
-  </si>
-  <si>
-    <t>Product</t>
-  </si>
-  <si>
-    <t>Laptop</t>
-  </si>
-  <si>
-    <t>Mobile</t>
-  </si>
-  <si>
-    <t>Camera</t>
-  </si>
-  <si>
-    <t>Tablet</t>
-  </si>
-  <si>
-    <t>Monitor</t>
-  </si>
-  <si>
-    <t>Salesperson</t>
-  </si>
-  <si>
-    <t>Pallavi Desai</t>
-  </si>
-  <si>
-    <t>Simran Kaur</t>
-  </si>
-  <si>
-    <t>Sahana Murthy</t>
-  </si>
-  <si>
-    <t>Gayatri Joshi</t>
-  </si>
-  <si>
-    <t>Sanjay Patel</t>
-  </si>
-  <si>
-    <t>Day</t>
-  </si>
-  <si>
-    <t>Month</t>
-  </si>
-  <si>
-    <t>2026-01</t>
-  </si>
-  <si>
-    <t>2026-02</t>
-  </si>
-  <si>
-    <t>2026-03</t>
-  </si>
-</sst>
-</file>
-
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="1">
-    <numFmt numFmtId="164" formatCode="yyyy\-mm\-dd"/>
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <numFmts count="2">
+    <numFmt numFmtId="164" formatCode="yyyy-mm-dd"/>
+    <numFmt numFmtId="165" formatCode="YYYY-MM-DD"/>
   </numFmts>
-  <fonts count="1" x14ac:knownFonts="1">
+  <fonts count="1">
     <font>
-      <sz val="11"/>
-      <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
+      <color theme="1"/>
+      <sz val="11"/>
       <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="2">
     <fill>
-      <patternFill patternType="none"/>
+      <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
@@ -157,22 +55,81 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
   <cellXfs count="2">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Normal" xfId="0" builtinId="0"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
   </cellStyles>
-  <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
-  <extLst>
-    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
-      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
-    </ext>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
-      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
-    </ext>
-  </extLst>
+  <colors>
+    <indexedColors>
+      <rgbColor rgb="00000000"/>
+      <rgbColor rgb="00FFFFFF"/>
+      <rgbColor rgb="00FF0000"/>
+      <rgbColor rgb="0000FF00"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00000000"/>
+      <rgbColor rgb="00FFFFFF"/>
+      <rgbColor rgb="00FF0000"/>
+      <rgbColor rgb="0000FF00"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00800000"/>
+      <rgbColor rgb="00008000"/>
+      <rgbColor rgb="00000080"/>
+      <rgbColor rgb="00808000"/>
+      <rgbColor rgb="00800080"/>
+      <rgbColor rgb="00008080"/>
+      <rgbColor rgb="00C0C0C0"/>
+      <rgbColor rgb="00808080"/>
+      <rgbColor rgb="009999FF"/>
+      <rgbColor rgb="00993366"/>
+      <rgbColor rgb="00FFFFCC"/>
+      <rgbColor rgb="00CCFFFF"/>
+      <rgbColor rgb="00660066"/>
+      <rgbColor rgb="00FF8080"/>
+      <rgbColor rgb="000066CC"/>
+      <rgbColor rgb="00CCCCFF"/>
+      <rgbColor rgb="00000080"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00800080"/>
+      <rgbColor rgb="00800000"/>
+      <rgbColor rgb="00008080"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="0000CCFF"/>
+      <rgbColor rgb="00CCFFFF"/>
+      <rgbColor rgb="00CCFFCC"/>
+      <rgbColor rgb="00FFFF99"/>
+      <rgbColor rgb="0099CCFF"/>
+      <rgbColor rgb="00FF99CC"/>
+      <rgbColor rgb="00CC99FF"/>
+      <rgbColor rgb="00FFCC99"/>
+      <rgbColor rgb="003366FF"/>
+      <rgbColor rgb="0033CCCC"/>
+      <rgbColor rgb="0099CC00"/>
+      <rgbColor rgb="00FFCC00"/>
+      <rgbColor rgb="00FF9900"/>
+      <rgbColor rgb="00FF6600"/>
+      <rgbColor rgb="00666699"/>
+      <rgbColor rgb="00969696"/>
+      <rgbColor rgb="00003366"/>
+      <rgbColor rgb="00339966"/>
+      <rgbColor rgb="00003300"/>
+      <rgbColor rgb="00333300"/>
+      <rgbColor rgb="00993300"/>
+      <rgbColor rgb="00993366"/>
+      <rgbColor rgb="00333399"/>
+      <rgbColor rgb="00333333"/>
+    </indexedColors>
+  </colors>
 </styleSheet>
 </file>
 
@@ -460,43 +417,53 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:B4"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
-  <cols>
-    <col min="1" max="1" width="38.85546875" customWidth="1"/>
-    <col min="2" max="2" width="51.28515625" customWidth="1"/>
-  </cols>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" t="s">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A2" t="s">
-        <v>2</v>
-      </c>
-      <c r="B2">
-        <v>657182734.13143659</v>
-      </c>
-    </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A3" t="s">
-        <v>3</v>
-      </c>
-      <c r="B3">
-        <v>55352.729412943299</v>
-      </c>
-    </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A4" t="s">
-        <v>4</v>
-      </c>
-      <c r="B4">
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>Metric</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>Value</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Total Revenue</t>
+        </is>
+      </c>
+      <c r="B2" t="n">
+        <v>657182734.1314366</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Total Quantity Sold</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
+        <v>55352.7294129433</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Unique Orders</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
         <v>9982</v>
       </c>
     </row>
@@ -506,91 +473,113 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:D6"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A1" t="s">
-        <v>5</v>
-      </c>
-      <c r="B1" t="s">
-        <v>6</v>
-      </c>
-      <c r="C1" t="s">
-        <v>7</v>
-      </c>
-      <c r="D1" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A2" t="s">
-        <v>9</v>
-      </c>
-      <c r="B2">
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>Region</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>Total_Revenue</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>Total_Quantity</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>Total_Orders</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>West</t>
+        </is>
+      </c>
+      <c r="B2" t="n">
         <v>167372900</v>
       </c>
-      <c r="C2">
+      <c r="C2" t="n">
         <v>14068</v>
       </c>
-      <c r="D2">
+      <c r="D2" t="n">
         <v>2534</v>
       </c>
     </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A3" t="s">
-        <v>10</v>
-      </c>
-      <c r="B3">
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>East</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
         <v>165931240.0120216</v>
       </c>
-      <c r="C3">
+      <c r="C3" t="n">
         <v>14233.63764776598</v>
       </c>
-      <c r="D3">
+      <c r="D3" t="n">
         <v>2536</v>
       </c>
     </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A4" t="s">
-        <v>11</v>
-      </c>
-      <c r="B4">
-        <v>163684594.11941499</v>
-      </c>
-      <c r="C4">
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>North</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>163684594.119415</v>
+      </c>
+      <c r="C4" t="n">
         <v>13783.09176517732</v>
       </c>
-      <c r="D4">
+      <c r="D4" t="n">
         <v>2515</v>
       </c>
     </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A5" t="s">
-        <v>12</v>
-      </c>
-      <c r="B5">
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>South</t>
+        </is>
+      </c>
+      <c r="B5" t="n">
         <v>159843000</v>
       </c>
-      <c r="C5">
+      <c r="C5" t="n">
         <v>13250</v>
       </c>
-      <c r="D5">
+      <c r="D5" t="n">
         <v>2394</v>
       </c>
     </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A6" t="s">
-        <v>13</v>
-      </c>
-      <c r="B6">
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> south </t>
+        </is>
+      </c>
+      <c r="B6" t="n">
         <v>351000</v>
       </c>
-      <c r="C6">
+      <c r="C6" t="n">
         <v>18</v>
       </c>
-      <c r="D6">
+      <c r="D6" t="n">
         <v>3</v>
       </c>
     </row>
@@ -600,73 +589,93 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:C6"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A1" t="s">
-        <v>14</v>
-      </c>
-      <c r="B1" t="s">
-        <v>6</v>
-      </c>
-      <c r="C1" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A2" t="s">
-        <v>15</v>
-      </c>
-      <c r="B2">
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>Product</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>Total_Revenue</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>Total_Quantity</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Laptop</t>
+        </is>
+      </c>
+      <c r="B2" t="n">
         <v>219735000</v>
       </c>
-      <c r="C2">
+      <c r="C2" t="n">
         <v>4883</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A3" t="s">
-        <v>16</v>
-      </c>
-      <c r="B3">
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Mobile</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
         <v>96600000</v>
       </c>
-      <c r="C3">
+      <c r="C3" t="n">
         <v>4830</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A4" t="s">
-        <v>17</v>
-      </c>
-      <c r="B4">
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Camera</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
         <v>79291651.77319175</v>
       </c>
-      <c r="C4">
-        <v>4405.0917651773188</v>
-      </c>
-    </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A5" t="s">
-        <v>18</v>
-      </c>
-      <c r="B5">
-        <v>66473188.238829903</v>
-      </c>
-      <c r="C5">
-        <v>4438.5458825886599</v>
-      </c>
-    </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A6" t="s">
-        <v>19</v>
-      </c>
-      <c r="B6">
+      <c r="C4" t="n">
+        <v>4405.091765177319</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Tablet</t>
+        </is>
+      </c>
+      <c r="B5" t="n">
+        <v>66473188.2388299</v>
+      </c>
+      <c r="C5" t="n">
+        <v>4438.54588258866</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Monitor</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
         <v>54492000</v>
       </c>
-      <c r="C6">
+      <c r="C6" t="n">
         <v>4541</v>
       </c>
     </row>
@@ -676,73 +685,93 @@
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:C6"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A1" t="s">
-        <v>20</v>
-      </c>
-      <c r="B1" t="s">
-        <v>6</v>
-      </c>
-      <c r="C1" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A2" t="s">
-        <v>21</v>
-      </c>
-      <c r="B2">
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>Salesperson</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>Total_Revenue</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>Total_Orders</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Pallavi Desai</t>
+        </is>
+      </c>
+      <c r="B2" t="n">
         <v>13795500</v>
       </c>
-      <c r="C2">
+      <c r="C2" t="n">
         <v>211</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A3" t="s">
-        <v>22</v>
-      </c>
-      <c r="B3">
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Simran Kaur</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
         <v>12428600</v>
       </c>
-      <c r="C3">
+      <c r="C3" t="n">
         <v>209</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A4" t="s">
-        <v>23</v>
-      </c>
-      <c r="B4">
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Sahana Murthy</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
         <v>10888200</v>
       </c>
-      <c r="C4">
+      <c r="C4" t="n">
         <v>184</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A5" t="s">
-        <v>24</v>
-      </c>
-      <c r="B5">
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Gayatri Joshi</t>
+        </is>
+      </c>
+      <c r="B5" t="n">
         <v>10422900</v>
       </c>
-      <c r="C5">
+      <c r="C5" t="n">
         <v>181</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A6" t="s">
-        <v>25</v>
-      </c>
-      <c r="B6">
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Sanjay Patel</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
         <v>9666688.238829894</v>
       </c>
-      <c r="C6">
+      <c r="C6" t="n">
         <v>117</v>
       </c>
     </row>
@@ -752,1281 +781,1293 @@
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:D91"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A1" t="s">
-        <v>26</v>
-      </c>
-      <c r="B1" t="s">
-        <v>6</v>
-      </c>
-      <c r="C1" t="s">
-        <v>7</v>
-      </c>
-      <c r="D1" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A2" s="1">
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>Day</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>Total_Revenue</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>Total_Quantity</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>Total_Orders</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="1" t="n">
         <v>46023</v>
       </c>
-      <c r="B2">
+      <c r="B2" t="n">
         <v>7524500</v>
       </c>
-      <c r="C2">
+      <c r="C2" t="n">
         <v>581</v>
       </c>
-      <c r="D2">
+      <c r="D2" t="n">
         <v>105</v>
       </c>
     </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A3" s="1">
+    <row r="3">
+      <c r="A3" s="1" t="n">
         <v>46024</v>
       </c>
-      <c r="B3">
+      <c r="B3" t="n">
         <v>9272000</v>
       </c>
-      <c r="C3">
+      <c r="C3" t="n">
         <v>653</v>
       </c>
-      <c r="D3">
+      <c r="D3" t="n">
         <v>107</v>
       </c>
     </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A4" s="1">
+    <row r="4">
+      <c r="A4" s="1" t="n">
         <v>46025</v>
       </c>
-      <c r="B4">
+      <c r="B4" t="n">
         <v>4382900</v>
       </c>
-      <c r="C4">
+      <c r="C4" t="n">
         <v>472</v>
       </c>
-      <c r="D4">
+      <c r="D4" t="n">
         <v>91</v>
       </c>
     </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A5" s="1">
+    <row r="5">
+      <c r="A5" s="1" t="n">
         <v>46026</v>
       </c>
-      <c r="B5">
+      <c r="B5" t="n">
         <v>6114900</v>
       </c>
-      <c r="C5">
+      <c r="C5" t="n">
         <v>531</v>
       </c>
-      <c r="D5">
+      <c r="D5" t="n">
         <v>103</v>
       </c>
     </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A6" s="1">
+    <row r="6">
+      <c r="A6" s="1" t="n">
         <v>46027</v>
       </c>
-      <c r="B6">
+      <c r="B6" t="n">
         <v>7292700</v>
       </c>
-      <c r="C6">
+      <c r="C6" t="n">
         <v>610</v>
       </c>
-      <c r="D6">
+      <c r="D6" t="n">
         <v>109</v>
       </c>
     </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A7" s="1">
+    <row r="7">
+      <c r="A7" s="1" t="n">
         <v>46028</v>
       </c>
-      <c r="B7">
+      <c r="B7" t="n">
         <v>6989300</v>
       </c>
-      <c r="C7">
+      <c r="C7" t="n">
         <v>640</v>
       </c>
-      <c r="D7">
+      <c r="D7" t="n">
         <v>115</v>
       </c>
     </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A8" s="1">
+    <row r="8">
+      <c r="A8" s="1" t="n">
         <v>46029</v>
       </c>
-      <c r="B8">
+      <c r="B8" t="n">
         <v>8582300</v>
       </c>
-      <c r="C8">
+      <c r="C8" t="n">
         <v>522</v>
       </c>
-      <c r="D8">
+      <c r="D8" t="n">
         <v>97</v>
       </c>
     </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A9" s="1">
+    <row r="9">
+      <c r="A9" s="1" t="n">
         <v>46030</v>
       </c>
-      <c r="B9">
+      <c r="B9" t="n">
         <v>7590800</v>
       </c>
-      <c r="C9">
+      <c r="C9" t="n">
         <v>543</v>
       </c>
-      <c r="D9">
+      <c r="D9" t="n">
         <v>105</v>
       </c>
     </row>
-    <row r="10" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A10" s="1">
+    <row r="10">
+      <c r="A10" s="1" t="n">
         <v>46031</v>
       </c>
-      <c r="B10">
+      <c r="B10" t="n">
         <v>5763900</v>
       </c>
-      <c r="C10">
+      <c r="C10" t="n">
         <v>561</v>
       </c>
-      <c r="D10">
+      <c r="D10" t="n">
         <v>108</v>
       </c>
     </row>
-    <row r="11" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A11" s="1">
+    <row r="11">
+      <c r="A11" s="1" t="n">
         <v>46032</v>
       </c>
-      <c r="B11">
-        <v>6743825.8865958722</v>
-      </c>
-      <c r="C11">
-        <v>540.54588258865954</v>
-      </c>
-      <c r="D11">
+      <c r="B11" t="n">
+        <v>6743825.886595872</v>
+      </c>
+      <c r="C11" t="n">
+        <v>540.5458825886595</v>
+      </c>
+      <c r="D11" t="n">
         <v>98</v>
       </c>
     </row>
-    <row r="12" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A12" s="1">
+    <row r="12">
+      <c r="A12" s="1" t="n">
         <v>46033</v>
       </c>
-      <c r="B12">
+      <c r="B12" t="n">
         <v>8682000</v>
       </c>
-      <c r="C12">
+      <c r="C12" t="n">
         <v>630</v>
       </c>
-      <c r="D12">
+      <c r="D12" t="n">
         <v>116</v>
       </c>
     </row>
-    <row r="13" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A13" s="1">
+    <row r="13">
+      <c r="A13" s="1" t="n">
         <v>46034</v>
       </c>
-      <c r="B13">
+      <c r="B13" t="n">
         <v>7966200</v>
       </c>
-      <c r="C13">
+      <c r="C13" t="n">
         <v>651</v>
       </c>
-      <c r="D13">
+      <c r="D13" t="n">
         <v>110</v>
       </c>
     </row>
-    <row r="14" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A14" s="1">
+    <row r="14">
+      <c r="A14" s="1" t="n">
         <v>46035</v>
       </c>
-      <c r="B14">
+      <c r="B14" t="n">
         <v>7553100</v>
       </c>
-      <c r="C14">
+      <c r="C14" t="n">
         <v>697</v>
       </c>
-      <c r="D14">
+      <c r="D14" t="n">
         <v>125</v>
       </c>
     </row>
-    <row r="15" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A15" s="1">
+    <row r="15">
+      <c r="A15" s="1" t="n">
         <v>46036</v>
       </c>
-      <c r="B15">
+      <c r="B15" t="n">
         <v>5483764.706471649</v>
       </c>
-      <c r="C15">
-        <v>530.54588258865954</v>
-      </c>
-      <c r="D15">
+      <c r="C15" t="n">
+        <v>530.5458825886595</v>
+      </c>
+      <c r="D15" t="n">
         <v>90</v>
       </c>
     </row>
-    <row r="16" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A16" s="1">
+    <row r="16">
+      <c r="A16" s="1" t="n">
         <v>46037</v>
       </c>
-      <c r="B16">
+      <c r="B16" t="n">
         <v>5675100</v>
       </c>
-      <c r="C16">
+      <c r="C16" t="n">
         <v>538</v>
       </c>
-      <c r="D16">
+      <c r="D16" t="n">
         <v>92</v>
       </c>
     </row>
-    <row r="17" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A17" s="1">
+    <row r="17">
+      <c r="A17" s="1" t="n">
         <v>46038</v>
       </c>
-      <c r="B17">
+      <c r="B17" t="n">
         <v>5060800</v>
       </c>
-      <c r="C17">
+      <c r="C17" t="n">
         <v>463</v>
       </c>
-      <c r="D17">
+      <c r="D17" t="n">
         <v>89</v>
       </c>
     </row>
-    <row r="18" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A18" s="1">
+    <row r="18">
+      <c r="A18" s="1" t="n">
         <v>46039</v>
       </c>
-      <c r="B18">
+      <c r="B18" t="n">
         <v>9960100</v>
       </c>
-      <c r="C18">
+      <c r="C18" t="n">
         <v>676</v>
       </c>
-      <c r="D18">
+      <c r="D18" t="n">
         <v>117</v>
       </c>
     </row>
-    <row r="19" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A19" s="1">
+    <row r="19">
+      <c r="A19" s="1" t="n">
         <v>46040</v>
       </c>
-      <c r="B19">
+      <c r="B19" t="n">
         <v>6935600</v>
       </c>
-      <c r="C19">
+      <c r="C19" t="n">
         <v>571</v>
       </c>
-      <c r="D19">
+      <c r="D19" t="n">
         <v>103</v>
       </c>
     </row>
-    <row r="20" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A20" s="1">
+    <row r="20">
+      <c r="A20" s="1" t="n">
         <v>46041</v>
       </c>
-      <c r="B20">
+      <c r="B20" t="n">
         <v>7487200</v>
       </c>
-      <c r="C20">
+      <c r="C20" t="n">
         <v>659</v>
       </c>
-      <c r="D20">
+      <c r="D20" t="n">
         <v>114</v>
       </c>
     </row>
-    <row r="21" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A21" s="1">
+    <row r="21">
+      <c r="A21" s="1" t="n">
         <v>46042</v>
       </c>
-      <c r="B21">
+      <c r="B21" t="n">
         <v>6045200</v>
       </c>
-      <c r="C21">
+      <c r="C21" t="n">
         <v>606</v>
       </c>
-      <c r="D21">
+      <c r="D21" t="n">
         <v>119</v>
       </c>
     </row>
-    <row r="22" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A22" s="1">
+    <row r="22">
+      <c r="A22" s="1" t="n">
         <v>46043</v>
       </c>
-      <c r="B22">
+      <c r="B22" t="n">
         <v>7431000</v>
       </c>
-      <c r="C22">
+      <c r="C22" t="n">
         <v>688</v>
       </c>
-      <c r="D22">
+      <c r="D22" t="n">
         <v>126</v>
       </c>
     </row>
-    <row r="23" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A23" s="1">
+    <row r="23">
+      <c r="A23" s="1" t="n">
         <v>46044</v>
       </c>
-      <c r="B23">
+      <c r="B23" t="n">
         <v>4540500</v>
       </c>
-      <c r="C23">
+      <c r="C23" t="n">
         <v>456</v>
       </c>
-      <c r="D23">
+      <c r="D23" t="n">
         <v>87</v>
       </c>
     </row>
-    <row r="24" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A24" s="1">
+    <row r="24">
+      <c r="A24" s="1" t="n">
         <v>46045</v>
       </c>
-      <c r="B24">
+      <c r="B24" t="n">
         <v>5132600</v>
       </c>
-      <c r="C24">
+      <c r="C24" t="n">
         <v>549</v>
       </c>
-      <c r="D24">
+      <c r="D24" t="n">
         <v>111</v>
       </c>
     </row>
-    <row r="25" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A25" s="1">
+    <row r="25">
+      <c r="A25" s="1" t="n">
         <v>46046</v>
       </c>
-      <c r="B25">
+      <c r="B25" t="n">
         <v>7059800</v>
       </c>
-      <c r="C25">
+      <c r="C25" t="n">
         <v>591</v>
       </c>
-      <c r="D25">
+      <c r="D25" t="n">
         <v>110</v>
       </c>
     </row>
-    <row r="26" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A26" s="1">
+    <row r="26">
+      <c r="A26" s="1" t="n">
         <v>46047</v>
       </c>
-      <c r="B26">
+      <c r="B26" t="n">
         <v>10224700</v>
       </c>
-      <c r="C26">
+      <c r="C26" t="n">
         <v>715</v>
       </c>
-      <c r="D26">
+      <c r="D26" t="n">
         <v>127</v>
       </c>
     </row>
-    <row r="27" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A27" s="1">
+    <row r="27">
+      <c r="A27" s="1" t="n">
         <v>46048</v>
       </c>
-      <c r="B27">
+      <c r="B27" t="n">
         <v>8719629.412943298</v>
       </c>
-      <c r="C27">
-        <v>628.54588258865954</v>
-      </c>
-      <c r="D27">
+      <c r="C27" t="n">
+        <v>628.5458825886595</v>
+      </c>
+      <c r="D27" t="n">
         <v>115</v>
       </c>
     </row>
-    <row r="28" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A28" s="1">
+    <row r="28">
+      <c r="A28" s="1" t="n">
         <v>46049</v>
       </c>
-      <c r="B28">
+      <c r="B28" t="n">
         <v>5859200</v>
       </c>
-      <c r="C28">
+      <c r="C28" t="n">
         <v>603</v>
       </c>
-      <c r="D28">
+      <c r="D28" t="n">
         <v>112</v>
       </c>
     </row>
-    <row r="29" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A29" s="1">
+    <row r="29">
+      <c r="A29" s="1" t="n">
         <v>46050</v>
       </c>
-      <c r="B29">
+      <c r="B29" t="n">
         <v>8402200</v>
       </c>
-      <c r="C29">
+      <c r="C29" t="n">
         <v>634</v>
       </c>
-      <c r="D29">
+      <c r="D29" t="n">
         <v>126</v>
       </c>
     </row>
-    <row r="30" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A30" s="1">
+    <row r="30">
+      <c r="A30" s="1" t="n">
         <v>46051</v>
       </c>
-      <c r="B30">
+      <c r="B30" t="n">
         <v>3740500</v>
       </c>
-      <c r="C30">
+      <c r="C30" t="n">
         <v>411</v>
       </c>
-      <c r="D30">
+      <c r="D30" t="n">
         <v>77</v>
       </c>
     </row>
-    <row r="31" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A31" s="1">
+    <row r="31">
+      <c r="A31" s="1" t="n">
         <v>46052</v>
       </c>
-      <c r="B31">
+      <c r="B31" t="n">
         <v>9027200</v>
       </c>
-      <c r="C31">
+      <c r="C31" t="n">
         <v>771</v>
       </c>
-      <c r="D31">
+      <c r="D31" t="n">
         <v>125</v>
       </c>
     </row>
-    <row r="32" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A32" s="1">
+    <row r="32">
+      <c r="A32" s="1" t="n">
         <v>46053</v>
       </c>
-      <c r="B32">
+      <c r="B32" t="n">
         <v>6984200</v>
       </c>
-      <c r="C32">
+      <c r="C32" t="n">
         <v>571</v>
       </c>
-      <c r="D32">
+      <c r="D32" t="n">
         <v>100</v>
       </c>
     </row>
-    <row r="33" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A33" s="1">
+    <row r="33">
+      <c r="A33" s="1" t="n">
         <v>46054</v>
       </c>
-      <c r="B33">
+      <c r="B33" t="n">
         <v>7007400</v>
       </c>
-      <c r="C33">
+      <c r="C33" t="n">
         <v>633</v>
       </c>
-      <c r="D33">
+      <c r="D33" t="n">
         <v>106</v>
       </c>
     </row>
-    <row r="34" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A34" s="1">
+    <row r="34">
+      <c r="A34" s="1" t="n">
         <v>46055</v>
       </c>
-      <c r="B34">
+      <c r="B34" t="n">
         <v>8133400</v>
       </c>
-      <c r="C34">
+      <c r="C34" t="n">
         <v>730</v>
       </c>
-      <c r="D34">
+      <c r="D34" t="n">
         <v>122</v>
       </c>
     </row>
-    <row r="35" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A35" s="1">
+    <row r="35">
+      <c r="A35" s="1" t="n">
         <v>46056</v>
       </c>
-      <c r="B35">
+      <c r="B35" t="n">
         <v>9059900</v>
       </c>
-      <c r="C35">
+      <c r="C35" t="n">
         <v>646</v>
       </c>
-      <c r="D35">
+      <c r="D35" t="n">
         <v>113</v>
       </c>
     </row>
-    <row r="36" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A36" s="1">
+    <row r="36">
+      <c r="A36" s="1" t="n">
         <v>46057</v>
       </c>
-      <c r="B36">
+      <c r="B36" t="n">
         <v>8075400</v>
       </c>
-      <c r="C36">
+      <c r="C36" t="n">
         <v>643</v>
       </c>
-      <c r="D36">
+      <c r="D36" t="n">
         <v>117</v>
       </c>
     </row>
-    <row r="37" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A37" s="1">
+    <row r="37">
+      <c r="A37" s="1" t="n">
         <v>46058</v>
       </c>
-      <c r="B37">
+      <c r="B37" t="n">
         <v>7154200</v>
       </c>
-      <c r="C37">
+      <c r="C37" t="n">
         <v>639</v>
       </c>
-      <c r="D37">
+      <c r="D37" t="n">
         <v>109</v>
       </c>
     </row>
-    <row r="38" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A38" s="1">
+    <row r="38">
+      <c r="A38" s="1" t="n">
         <v>46059</v>
       </c>
-      <c r="B38">
+      <c r="B38" t="n">
         <v>6550000</v>
       </c>
-      <c r="C38">
+      <c r="C38" t="n">
         <v>544</v>
       </c>
-      <c r="D38">
+      <c r="D38" t="n">
         <v>101</v>
       </c>
     </row>
-    <row r="39" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A39" s="1">
+    <row r="39">
+      <c r="A39" s="1" t="n">
         <v>46060</v>
       </c>
-      <c r="B39">
+      <c r="B39" t="n">
         <v>6324000</v>
       </c>
-      <c r="C39">
+      <c r="C39" t="n">
         <v>567</v>
       </c>
-      <c r="D39">
+      <c r="D39" t="n">
         <v>105</v>
       </c>
     </row>
-    <row r="40" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A40" s="1">
+    <row r="40">
+      <c r="A40" s="1" t="n">
         <v>46061</v>
       </c>
-      <c r="B40">
+      <c r="B40" t="n">
         <v>6606200</v>
       </c>
-      <c r="C40">
+      <c r="C40" t="n">
         <v>624</v>
       </c>
-      <c r="D40">
+      <c r="D40" t="n">
         <v>114</v>
       </c>
     </row>
-    <row r="41" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A41" s="1">
+    <row r="41">
+      <c r="A41" s="1" t="n">
         <v>46062</v>
       </c>
-      <c r="B41">
+      <c r="B41" t="n">
         <v>6923700</v>
       </c>
-      <c r="C41">
+      <c r="C41" t="n">
         <v>583</v>
       </c>
-      <c r="D41">
+      <c r="D41" t="n">
         <v>105</v>
       </c>
     </row>
-    <row r="42" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A42" s="1">
+    <row r="42">
+      <c r="A42" s="1" t="n">
         <v>46063</v>
       </c>
-      <c r="B42">
+      <c r="B42" t="n">
         <v>7356800</v>
       </c>
-      <c r="C42">
+      <c r="C42" t="n">
         <v>608</v>
       </c>
-      <c r="D42">
+      <c r="D42" t="n">
         <v>102</v>
       </c>
     </row>
-    <row r="43" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A43" s="1">
+    <row r="43">
+      <c r="A43" s="1" t="n">
         <v>46064</v>
       </c>
-      <c r="B43">
+      <c r="B43" t="n">
         <v>7912600</v>
       </c>
-      <c r="C43">
+      <c r="C43" t="n">
         <v>641</v>
       </c>
-      <c r="D43">
+      <c r="D43" t="n">
         <v>115</v>
       </c>
     </row>
-    <row r="44" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A44" s="1">
+    <row r="44">
+      <c r="A44" s="1" t="n">
         <v>46065</v>
       </c>
-      <c r="B44">
+      <c r="B44" t="n">
         <v>7653600</v>
       </c>
-      <c r="C44">
+      <c r="C44" t="n">
         <v>578</v>
       </c>
-      <c r="D44">
+      <c r="D44" t="n">
         <v>110</v>
       </c>
     </row>
-    <row r="45" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A45" s="1">
+    <row r="45">
+      <c r="A45" s="1" t="n">
         <v>46066</v>
       </c>
-      <c r="B45">
+      <c r="B45" t="n">
         <v>6410200</v>
       </c>
-      <c r="C45">
+      <c r="C45" t="n">
         <v>590</v>
       </c>
-      <c r="D45">
+      <c r="D45" t="n">
         <v>108</v>
       </c>
     </row>
-    <row r="46" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A46" s="1">
+    <row r="46">
+      <c r="A46" s="1" t="n">
         <v>46067</v>
       </c>
-      <c r="B46">
+      <c r="B46" t="n">
         <v>6329900</v>
       </c>
-      <c r="C46">
+      <c r="C46" t="n">
         <v>547</v>
       </c>
-      <c r="D46">
+      <c r="D46" t="n">
         <v>98</v>
       </c>
     </row>
-    <row r="47" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A47" s="1">
+    <row r="47">
+      <c r="A47" s="1" t="n">
         <v>46068</v>
       </c>
-      <c r="B47">
+      <c r="B47" t="n">
         <v>10982900</v>
       </c>
-      <c r="C47">
+      <c r="C47" t="n">
         <v>770</v>
       </c>
-      <c r="D47">
+      <c r="D47" t="n">
         <v>136</v>
       </c>
     </row>
-    <row r="48" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A48" s="1">
+    <row r="48">
+      <c r="A48" s="1" t="n">
         <v>46069</v>
       </c>
-      <c r="B48">
+      <c r="B48" t="n">
         <v>7365800</v>
       </c>
-      <c r="C48">
+      <c r="C48" t="n">
         <v>634</v>
       </c>
-      <c r="D48">
+      <c r="D48" t="n">
         <v>111</v>
       </c>
     </row>
-    <row r="49" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A49" s="1">
+    <row r="49">
+      <c r="A49" s="1" t="n">
         <v>46070</v>
       </c>
-      <c r="B49">
+      <c r="B49" t="n">
         <v>6191700</v>
       </c>
-      <c r="C49">
+      <c r="C49" t="n">
         <v>693</v>
       </c>
-      <c r="D49">
+      <c r="D49" t="n">
         <v>129</v>
       </c>
     </row>
-    <row r="50" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A50" s="1">
+    <row r="50">
+      <c r="A50" s="1" t="n">
         <v>46071</v>
       </c>
-      <c r="B50">
+      <c r="B50" t="n">
         <v>7907300</v>
       </c>
-      <c r="C50">
+      <c r="C50" t="n">
         <v>629</v>
       </c>
-      <c r="D50">
+      <c r="D50" t="n">
         <v>119</v>
       </c>
     </row>
-    <row r="51" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A51" s="1">
+    <row r="51">
+      <c r="A51" s="1" t="n">
         <v>46072</v>
       </c>
-      <c r="B51">
+      <c r="B51" t="n">
         <v>6227400</v>
       </c>
-      <c r="C51">
+      <c r="C51" t="n">
         <v>595</v>
       </c>
-      <c r="D51">
+      <c r="D51" t="n">
         <v>109</v>
       </c>
     </row>
-    <row r="52" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A52" s="1">
+    <row r="52">
+      <c r="A52" s="1" t="n">
         <v>46073</v>
       </c>
-      <c r="B52">
+      <c r="B52" t="n">
         <v>6723100</v>
       </c>
-      <c r="C52">
+      <c r="C52" t="n">
         <v>558</v>
       </c>
-      <c r="D52">
+      <c r="D52" t="n">
         <v>106</v>
       </c>
     </row>
-    <row r="53" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A53" s="1">
+    <row r="53">
+      <c r="A53" s="1" t="n">
         <v>46074</v>
       </c>
-      <c r="B53">
+      <c r="B53" t="n">
         <v>7022300</v>
       </c>
-      <c r="C53">
+      <c r="C53" t="n">
         <v>595</v>
       </c>
-      <c r="D53">
+      <c r="D53" t="n">
         <v>105</v>
       </c>
     </row>
-    <row r="54" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A54" s="1">
+    <row r="54">
+      <c r="A54" s="1" t="n">
         <v>46075</v>
       </c>
-      <c r="B54">
+      <c r="B54" t="n">
         <v>6712900</v>
       </c>
-      <c r="C54">
+      <c r="C54" t="n">
         <v>630</v>
       </c>
-      <c r="D54">
+      <c r="D54" t="n">
         <v>111</v>
       </c>
     </row>
-    <row r="55" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A55" s="1">
+    <row r="55">
+      <c r="A55" s="1" t="n">
         <v>46076</v>
       </c>
-      <c r="B55">
+      <c r="B55" t="n">
         <v>7784500</v>
       </c>
-      <c r="C55">
+      <c r="C55" t="n">
         <v>657</v>
       </c>
-      <c r="D55">
+      <c r="D55" t="n">
         <v>114</v>
       </c>
     </row>
-    <row r="56" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A56" s="1">
+    <row r="56">
+      <c r="A56" s="1" t="n">
         <v>46077</v>
       </c>
-      <c r="B56">
+      <c r="B56" t="n">
         <v>7010800</v>
       </c>
-      <c r="C56">
+      <c r="C56" t="n">
         <v>622</v>
       </c>
-      <c r="D56">
+      <c r="D56" t="n">
         <v>115</v>
       </c>
     </row>
-    <row r="57" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A57" s="1">
+    <row r="57">
+      <c r="A57" s="1" t="n">
         <v>46078</v>
       </c>
-      <c r="B57">
+      <c r="B57" t="n">
         <v>7850400</v>
       </c>
-      <c r="C57">
+      <c r="C57" t="n">
         <v>639</v>
       </c>
-      <c r="D57">
+      <c r="D57" t="n">
         <v>110</v>
       </c>
     </row>
-    <row r="58" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A58" s="1">
+    <row r="58">
+      <c r="A58" s="1" t="n">
         <v>46079</v>
       </c>
-      <c r="B58">
+      <c r="B58" t="n">
         <v>5571500</v>
       </c>
-      <c r="C58">
+      <c r="C58" t="n">
         <v>583</v>
       </c>
-      <c r="D58">
+      <c r="D58" t="n">
         <v>107</v>
       </c>
     </row>
-    <row r="59" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A59" s="1">
+    <row r="59">
+      <c r="A59" s="1" t="n">
         <v>46080</v>
       </c>
-      <c r="B59">
+      <c r="B59" t="n">
         <v>6429800</v>
       </c>
-      <c r="C59">
+      <c r="C59" t="n">
         <v>554</v>
       </c>
-      <c r="D59">
+      <c r="D59" t="n">
         <v>105</v>
       </c>
     </row>
-    <row r="60" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A60" s="1">
+    <row r="60">
+      <c r="A60" s="1" t="n">
         <v>46081</v>
       </c>
-      <c r="B60">
+      <c r="B60" t="n">
         <v>8377000</v>
       </c>
-      <c r="C60">
+      <c r="C60" t="n">
         <v>590</v>
       </c>
-      <c r="D60">
+      <c r="D60" t="n">
         <v>110</v>
       </c>
     </row>
-    <row r="61" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A61" s="1">
+    <row r="61">
+      <c r="A61" s="1" t="n">
         <v>46082</v>
       </c>
-      <c r="B61">
+      <c r="B61" t="n">
         <v>6221700</v>
       </c>
-      <c r="C61">
+      <c r="C61" t="n">
         <v>616</v>
       </c>
-      <c r="D61">
+      <c r="D61" t="n">
         <v>117</v>
       </c>
     </row>
-    <row r="62" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A62" s="1">
+    <row r="62">
+      <c r="A62" s="1" t="n">
         <v>46083</v>
       </c>
-      <c r="B62">
+      <c r="B62" t="n">
         <v>8438300</v>
       </c>
-      <c r="C62">
+      <c r="C62" t="n">
         <v>673</v>
       </c>
-      <c r="D62">
+      <c r="D62" t="n">
         <v>123</v>
       </c>
     </row>
-    <row r="63" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A63" s="1">
+    <row r="63">
+      <c r="A63" s="1" t="n">
         <v>46084</v>
       </c>
-      <c r="B63">
+      <c r="B63" t="n">
         <v>6000600</v>
       </c>
-      <c r="C63">
+      <c r="C63" t="n">
         <v>586</v>
       </c>
-      <c r="D63">
+      <c r="D63" t="n">
         <v>120</v>
       </c>
     </row>
-    <row r="64" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A64" s="1">
+    <row r="64">
+      <c r="A64" s="1" t="n">
         <v>46085</v>
       </c>
-      <c r="B64">
+      <c r="B64" t="n">
         <v>6011400</v>
       </c>
-      <c r="C64">
+      <c r="C64" t="n">
         <v>516</v>
       </c>
-      <c r="D64">
+      <c r="D64" t="n">
         <v>102</v>
       </c>
     </row>
-    <row r="65" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A65" s="1">
+    <row r="65">
+      <c r="A65" s="1" t="n">
         <v>46086</v>
       </c>
-      <c r="B65">
+      <c r="B65" t="n">
         <v>9539500</v>
       </c>
-      <c r="C65">
+      <c r="C65" t="n">
         <v>799</v>
       </c>
-      <c r="D65">
+      <c r="D65" t="n">
         <v>135</v>
       </c>
     </row>
-    <row r="66" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A66" s="1">
+    <row r="66">
+      <c r="A66" s="1" t="n">
         <v>46087</v>
       </c>
-      <c r="B66">
+      <c r="B66" t="n">
         <v>10270100</v>
       </c>
-      <c r="C66">
+      <c r="C66" t="n">
         <v>739</v>
       </c>
-      <c r="D66">
+      <c r="D66" t="n">
         <v>123</v>
       </c>
     </row>
-    <row r="67" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A67" s="1">
+    <row r="67">
+      <c r="A67" s="1" t="n">
         <v>46088</v>
       </c>
-      <c r="B67">
+      <c r="B67" t="n">
         <v>7461400</v>
       </c>
-      <c r="C67">
+      <c r="C67" t="n">
         <v>694</v>
       </c>
-      <c r="D67">
+      <c r="D67" t="n">
         <v>118</v>
       </c>
     </row>
-    <row r="68" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A68" s="1">
+    <row r="68">
+      <c r="A68" s="1" t="n">
         <v>46089</v>
       </c>
-      <c r="B68">
+      <c r="B68" t="n">
         <v>6561000</v>
       </c>
-      <c r="C68">
+      <c r="C68" t="n">
         <v>608</v>
       </c>
-      <c r="D68">
+      <c r="D68" t="n">
         <v>109</v>
       </c>
     </row>
-    <row r="69" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A69" s="1">
+    <row r="69">
+      <c r="A69" s="1" t="n">
         <v>46090</v>
       </c>
-      <c r="B69">
+      <c r="B69" t="n">
         <v>6450800</v>
       </c>
-      <c r="C69">
+      <c r="C69" t="n">
         <v>564</v>
       </c>
-      <c r="D69">
+      <c r="D69" t="n">
         <v>109</v>
       </c>
     </row>
-    <row r="70" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A70" s="1">
+    <row r="70">
+      <c r="A70" s="1" t="n">
         <v>46091</v>
       </c>
-      <c r="B70">
+      <c r="B70" t="n">
         <v>8025300</v>
       </c>
-      <c r="C70">
+      <c r="C70" t="n">
         <v>696</v>
       </c>
-      <c r="D70">
+      <c r="D70" t="n">
         <v>123</v>
       </c>
     </row>
-    <row r="71" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A71" s="1">
+    <row r="71">
+      <c r="A71" s="1" t="n">
         <v>46092</v>
       </c>
-      <c r="B71">
+      <c r="B71" t="n">
         <v>6537200</v>
       </c>
-      <c r="C71">
+      <c r="C71" t="n">
         <v>626</v>
       </c>
-      <c r="D71">
+      <c r="D71" t="n">
         <v>114</v>
       </c>
     </row>
-    <row r="72" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A72" s="1">
+    <row r="72">
+      <c r="A72" s="1" t="n">
         <v>46093</v>
       </c>
-      <c r="B72">
+      <c r="B72" t="n">
         <v>8406800</v>
       </c>
-      <c r="C72">
+      <c r="C72" t="n">
         <v>643</v>
       </c>
-      <c r="D72">
+      <c r="D72" t="n">
         <v>114</v>
       </c>
     </row>
-    <row r="73" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A73" s="1">
+    <row r="73">
+      <c r="A73" s="1" t="n">
         <v>46094</v>
       </c>
-      <c r="B73">
+      <c r="B73" t="n">
         <v>8258000</v>
       </c>
-      <c r="C73">
+      <c r="C73" t="n">
         <v>642</v>
       </c>
-      <c r="D73">
+      <c r="D73" t="n">
         <v>125</v>
       </c>
     </row>
-    <row r="74" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A74" s="1">
+    <row r="74">
+      <c r="A74" s="1" t="n">
         <v>46095</v>
       </c>
-      <c r="B74">
+      <c r="B74" t="n">
         <v>8373200</v>
       </c>
-      <c r="C74">
+      <c r="C74" t="n">
         <v>710</v>
       </c>
-      <c r="D74">
+      <c r="D74" t="n">
         <v>117</v>
       </c>
     </row>
-    <row r="75" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A75" s="1">
+    <row r="75">
+      <c r="A75" s="1" t="n">
         <v>46096</v>
       </c>
-      <c r="B75">
+      <c r="B75" t="n">
         <v>9070700</v>
       </c>
-      <c r="C75">
+      <c r="C75" t="n">
         <v>784</v>
       </c>
-      <c r="D75">
+      <c r="D75" t="n">
         <v>132</v>
       </c>
     </row>
-    <row r="76" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A76" s="1">
+    <row r="76">
+      <c r="A76" s="1" t="n">
         <v>46097</v>
       </c>
-      <c r="B76">
+      <c r="B76" t="n">
         <v>6059700</v>
       </c>
-      <c r="C76">
+      <c r="C76" t="n">
         <v>563</v>
       </c>
-      <c r="D76">
+      <c r="D76" t="n">
         <v>103</v>
       </c>
     </row>
-    <row r="77" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A77" s="1">
+    <row r="77">
+      <c r="A77" s="1" t="n">
         <v>46098</v>
       </c>
-      <c r="B77">
+      <c r="B77" t="n">
         <v>5546600</v>
       </c>
-      <c r="C77">
+      <c r="C77" t="n">
         <v>552</v>
       </c>
-      <c r="D77">
+      <c r="D77" t="n">
         <v>107</v>
       </c>
     </row>
-    <row r="78" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A78" s="1">
+    <row r="78">
+      <c r="A78" s="1" t="n">
         <v>46099</v>
       </c>
-      <c r="B78">
+      <c r="B78" t="n">
         <v>8214000</v>
       </c>
-      <c r="C78">
+      <c r="C78" t="n">
         <v>652</v>
       </c>
-      <c r="D78">
+      <c r="D78" t="n">
         <v>112</v>
       </c>
     </row>
-    <row r="79" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A79" s="1">
+    <row r="79">
+      <c r="A79" s="1" t="n">
         <v>46100</v>
       </c>
-      <c r="B79">
+      <c r="B79" t="n">
         <v>5926100</v>
       </c>
-      <c r="C79">
+      <c r="C79" t="n">
         <v>615</v>
       </c>
-      <c r="D79">
+      <c r="D79" t="n">
         <v>114</v>
       </c>
     </row>
-    <row r="80" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A80" s="1">
+    <row r="80">
+      <c r="A80" s="1" t="n">
         <v>46101</v>
       </c>
-      <c r="B80">
+      <c r="B80" t="n">
         <v>9673400</v>
       </c>
-      <c r="C80">
+      <c r="C80" t="n">
         <v>651</v>
       </c>
-      <c r="D80">
+      <c r="D80" t="n">
         <v>124</v>
       </c>
     </row>
-    <row r="81" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A81" s="1">
+    <row r="81">
+      <c r="A81" s="1" t="n">
         <v>46102</v>
       </c>
-      <c r="B81">
-        <v>7722025.8865958722</v>
-      </c>
-      <c r="C81">
-        <v>656.54588258865954</v>
-      </c>
-      <c r="D81">
+      <c r="B81" t="n">
+        <v>7722025.886595872</v>
+      </c>
+      <c r="C81" t="n">
+        <v>656.5458825886595</v>
+      </c>
+      <c r="D81" t="n">
         <v>107</v>
       </c>
     </row>
-    <row r="82" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A82" s="1">
+    <row r="82">
+      <c r="A82" s="1" t="n">
         <v>46103</v>
       </c>
-      <c r="B82">
+      <c r="B82" t="n">
         <v>8583400</v>
       </c>
-      <c r="C82">
+      <c r="C82" t="n">
         <v>642</v>
       </c>
-      <c r="D82">
+      <c r="D82" t="n">
         <v>111</v>
       </c>
     </row>
-    <row r="83" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A83" s="1">
+    <row r="83">
+      <c r="A83" s="1" t="n">
         <v>46104</v>
       </c>
-      <c r="B83">
+      <c r="B83" t="n">
         <v>8097488.238829894</v>
       </c>
-      <c r="C83">
-        <v>605.54588258865954</v>
-      </c>
-      <c r="D83">
+      <c r="C83" t="n">
+        <v>605.5458825886595</v>
+      </c>
+      <c r="D83" t="n">
         <v>106</v>
       </c>
     </row>
-    <row r="84" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A84" s="1">
+    <row r="84">
+      <c r="A84" s="1" t="n">
         <v>46105</v>
       </c>
-      <c r="B84">
+      <c r="B84" t="n">
         <v>5290900</v>
       </c>
-      <c r="C84">
+      <c r="C84" t="n">
         <v>544</v>
       </c>
-      <c r="D84">
+      <c r="D84" t="n">
         <v>96</v>
       </c>
     </row>
-    <row r="85" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A85" s="1">
+    <row r="85">
+      <c r="A85" s="1" t="n">
         <v>46106</v>
       </c>
-      <c r="B85">
+      <c r="B85" t="n">
         <v>8583800</v>
       </c>
-      <c r="C85">
+      <c r="C85" t="n">
         <v>594</v>
       </c>
-      <c r="D85">
+      <c r="D85" t="n">
         <v>106</v>
       </c>
     </row>
-    <row r="86" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A86" s="1">
+    <row r="86">
+      <c r="A86" s="1" t="n">
         <v>46107</v>
       </c>
-      <c r="B86">
+      <c r="B86" t="n">
         <v>9752100</v>
       </c>
-      <c r="C86">
+      <c r="C86" t="n">
         <v>708</v>
       </c>
-      <c r="D86">
+      <c r="D86" t="n">
         <v>121</v>
       </c>
     </row>
-    <row r="87" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A87" s="1">
+    <row r="87">
+      <c r="A87" s="1" t="n">
         <v>46108</v>
       </c>
-      <c r="B87">
+      <c r="B87" t="n">
         <v>6783900</v>
       </c>
-      <c r="C87">
+      <c r="C87" t="n">
         <v>648</v>
       </c>
-      <c r="D87">
+      <c r="D87" t="n">
         <v>120</v>
       </c>
     </row>
-    <row r="88" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A88" s="1">
+    <row r="88">
+      <c r="A88" s="1" t="n">
         <v>46109</v>
       </c>
-      <c r="B88">
+      <c r="B88" t="n">
         <v>6331700</v>
       </c>
-      <c r="C88">
+      <c r="C88" t="n">
         <v>519</v>
       </c>
-      <c r="D88">
+      <c r="D88" t="n">
         <v>91</v>
       </c>
     </row>
-    <row r="89" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A89" s="1">
+    <row r="89">
+      <c r="A89" s="1" t="n">
         <v>46110</v>
       </c>
-      <c r="B89">
+      <c r="B89" t="n">
         <v>6763600</v>
       </c>
-      <c r="C89">
+      <c r="C89" t="n">
         <v>587</v>
       </c>
-      <c r="D89">
+      <c r="D89" t="n">
         <v>105</v>
       </c>
     </row>
-    <row r="90" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A90" s="1">
+    <row r="90">
+      <c r="A90" s="1" t="n">
         <v>46111</v>
       </c>
-      <c r="B90">
+      <c r="B90" t="n">
         <v>10085400</v>
       </c>
-      <c r="C90">
+      <c r="C90" t="n">
         <v>730</v>
       </c>
-      <c r="D90">
+      <c r="D90" t="n">
         <v>132</v>
       </c>
     </row>
-    <row r="91" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A91" s="1">
+    <row r="91">
+      <c r="A91" s="1" t="n">
         <v>46112</v>
       </c>
-      <c r="B91">
+      <c r="B91" t="n">
         <v>6145200</v>
       </c>
-      <c r="C91">
+      <c r="C91" t="n">
         <v>560</v>
       </c>
-      <c r="D91">
+      <c r="D91" t="n">
         <v>102</v>
       </c>
     </row>
@@ -2036,63 +2077,81 @@
 </file>
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0500-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:D4"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A1" t="s">
-        <v>27</v>
-      </c>
-      <c r="B1" t="s">
-        <v>6</v>
-      </c>
-      <c r="C1" t="s">
-        <v>7</v>
-      </c>
-      <c r="D1" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A2" t="s">
-        <v>28</v>
-      </c>
-      <c r="B2">
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>Month</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>Total_Revenue</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>Total_Quantity</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>Total_Orders</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>2026-01</t>
+        </is>
+      </c>
+      <c r="B2" t="n">
         <v>218227720.0060108</v>
       </c>
-      <c r="C2">
+      <c r="C2" t="n">
         <v>18292.63764776598</v>
       </c>
-      <c r="D2">
+      <c r="D2" t="n">
         <v>3329</v>
       </c>
     </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A3" t="s">
-        <v>29</v>
-      </c>
-      <c r="B3">
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>2026-02</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
         <v>203654700</v>
       </c>
-      <c r="C3">
+      <c r="C3" t="n">
         <v>17322</v>
       </c>
-      <c r="D3">
+      <c r="D3" t="n">
         <v>3112</v>
       </c>
     </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A4" t="s">
-        <v>30</v>
-      </c>
-      <c r="B4">
-        <v>235185314.12542579</v>
-      </c>
-      <c r="C4">
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>2026-03</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>235185314.1254258</v>
+      </c>
+      <c r="C4" t="n">
         <v>19723.09176517732</v>
       </c>
-      <c r="D4">
+      <c r="D4" t="n">
         <v>3538</v>
       </c>
     </row>

</xml_diff>